<commit_message>
📄 Update report documents and template tables
Updates:
- Updated Laporan Akhir Penelitian Malaria.docx
- Added PDF export: Laporan Akhir Penelitian Malaria.pdf
- Updated template tables (Table3-6) with latest format

Changes:
✓ Report documents updated
✓ PDF version added for easy sharing
✓ Template tables refreshed with correct formatting

Note: Temporary Excel files (~.xlsx) excluded from commit
</commit_message>
<xml_diff>
--- a/luaran/templates/tables/Table3_IML_Classification.xlsx
+++ b/luaran/templates/tables/Table3_IML_Classification.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IML Lifecycle" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="IML Lifecycle" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>